<commit_message>
Switch classifier to Apertus, add production pipeline and label mapping
</commit_message>
<xml_diff>
--- a/data/Final_TT_CB_Labels.xlsx
+++ b/data/Final_TT_CB_Labels.xlsx
@@ -8,14 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TRA237227\Documents\tt_cb_classifier\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EECAFF-406F-4420-8567-A2B18CEE4CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802D7EC2-FF1B-4E69-B42B-16378F2F5DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32550" yWindow="-4575" windowWidth="38700" windowHeight="15285" xr2:uid="{BAAF2764-207B-4C09-8789-88A61ED89364}"/>
+    <workbookView xWindow="27850" yWindow="-8830" windowWidth="28800" windowHeight="15410" activeTab="2" xr2:uid="{BAAF2764-207B-4C09-8789-88A61ED89364}"/>
   </bookViews>
   <sheets>
     <sheet name="Train" sheetId="2" r:id="rId1"/>
-    <sheet name="Test" sheetId="3" r:id="rId2"/>
+    <sheet name="Dev" sheetId="4" r:id="rId2"/>
+    <sheet name="Test" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Dev!$A$1:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Test!$A$1:$E$91</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="409">
   <si>
     <t>Partical Action</t>
   </si>
@@ -511,9 +516,6 @@
     <t>7F-07793.02.03</t>
   </si>
   <si>
-    <t>7F-08320.03.05</t>
-  </si>
-  <si>
     <t>UR_00868.01.01</t>
   </si>
   <si>
@@ -866,6 +868,405 @@
   </si>
   <si>
     <t>Working together with the local community</t>
+  </si>
+  <si>
+    <t>7F-05448.04</t>
+  </si>
+  <si>
+    <t>Bioculture and Climate Change</t>
+  </si>
+  <si>
+    <t>Bolivia is highly vulnerable to the effects of Climate Change, particularly in its regions of greater population density and poverty. Over two phases, the program has helped Bolivia to improve the resilience capacity of its most vulnerable communities, while in parallel building up and strengthening the public sectors capacity in this area. The third and final phase aims to consolidate the mechanisms put in place by the State to implement its climate change related policies at national and subnational levels.</t>
+  </si>
+  <si>
+    <t>7F-06524.03</t>
+  </si>
+  <si>
+    <t>Indo-Swiss Programme on Building Energy Efficiency (BEEP)</t>
+  </si>
+  <si>
+    <t>Globally buildings account for 35% of energy use and about 20% of GHG emissions. In India, buildings even consume 40% of all energy and cause 40% of CO 2 emissions. Phase 2 of BEEP has shown that 30-45% of energy savings are possible in India with marginal additional costs compared to the current way of constructing. Based on the achievements of the previous phase, Phase 3 will focus on mainstreaming and scaling-up energy efficient and thermally comfortable building design and on promoting the on-site use of renewable energy sources.</t>
+  </si>
+  <si>
+    <t>7F-06576.05.51</t>
+  </si>
+  <si>
+    <t>UN CC:Learn The One UN Climate Change Learning Partnership Phase V</t>
+  </si>
+  <si>
+    <t>UN CC:Learn is the partnership of key multilateral organizations assisting member states in designing and implementing learning to address climate change. It supports countries in developing national strategies and designs and promotes learning materials to strengthen human resources and skills for climate resilient-development and global climate literacy. Switzerlands focus therein is on further advancing the youth component and strengthening the sustainability aspects of the initiative.</t>
+  </si>
+  <si>
+    <t>7F-06587.03.51</t>
+  </si>
+  <si>
+    <t>7F-06685.05.51</t>
+  </si>
+  <si>
+    <t>Backstopping SDC Climate Change and Environment (CC&amp;E) Network</t>
+  </si>
+  <si>
+    <t>A climate smart development cooperation requires continuous knowledge management and a sound thematic expertise. The next phase of the Backstopping Support Mandate (BSM) will help to capitalize on SDCs key learnings, stimulate capacity building, foster mainstreaming and provide thematic support in the field of climate change and environment This will allow the SDC Climate Change and Environment Network and the Global Programme Climate Change (GPCCE) help improve the overall quality of SDCs operational activities in this thematic field.</t>
+  </si>
+  <si>
+    <t>7F-06742.01</t>
+  </si>
+  <si>
+    <t>Strengthening policy dialogue on DRR &amp; RR of Andean countries</t>
+  </si>
+  <si>
+    <t>The project aims at strengthening policy dialogue on Disaster Risk Reduction and Rapid Response among Andean countries in particular and within the Latin America countries in general. The participation of SDCs key partners in DRR and humanitarian events (e.g. the yearly Humanitarian Network and Partnership Week) will facilitate knowledge exchange, experience sharing and increased collaboration within the region. The project will further contribute to this by engaging in knowledge management supporting regional policy dialogue, and by financially contributing to specific events.</t>
+  </si>
+  <si>
+    <t>7F-06872.03</t>
+  </si>
+  <si>
+    <t>Nature Conservation Programme</t>
+  </si>
+  <si>
+    <t>Switzerland supports North Macedonia in sustainable management of natural resources through practical application of conservation measures in the Bregalnica region. In the exit phase, institutions and organizations will be further strengthened for an effective management of protected areas, introduction of payments for ecosystem services and implementation of measures set out in the national strategies. By promoting sustainably produced products and services, economic benefit for the local population will be generated.</t>
+  </si>
+  <si>
+    <t>7F-06990.04</t>
+  </si>
+  <si>
+    <t>Global Forums for Rural Advisory Services (GFRAS) and Young Professional in Agriculture and Rural Development (YPARD)</t>
+  </si>
+  <si>
+    <t>The COVID-19 crisis magnified existing inequalities. The people with less access to resilience mechanisms, such as the poor, women and youth groups are hardest hit, risking the loss of decades of improvement in poverty alleviation. Rural Advisory Services (RAS) are an important production input for millions of small farmers around the world. The two international networks based in Switzerland, and present in most geographical locations in the world will together develop and strengthen the ability of rural advisory services to better serve the smallholder farmers.</t>
+  </si>
+  <si>
+    <t>7F-07045.03.51</t>
+  </si>
+  <si>
+    <t>Gestión integral del agua</t>
+  </si>
+  <si>
+    <t>In Bolivia, Switzerland has been supporting the Ministry of the Environment and Water in improving integrated water and watershed management for several years. In this last phase of the project, support is given to the consolidation and implementation of the Plan Nacional de Cuencas (National Watershed Plan) to ensure water security and increase the climate resilience of vulnerable populations. Consolidation includes better coordination among various state levels, sectors and institutions and the systematization and capitalization of experiences and results.</t>
+  </si>
+  <si>
+    <t>7F-07182.01.51</t>
+  </si>
+  <si>
+    <t>Contribution to the Climate Action Accelerator (CAA)</t>
+  </si>
+  <si>
+    <t>The Climate Action Accelerator is a non-profit initiative that develops tools and solutions to support organisations of the aid, health and education sectors in reducing their carbon footprint. By the End of 2023, around 40 organisations (with a focus on Europe, Africa and South Asia) shall be engaged, and committed to oeuvre towards the decarbonisation of their own, and partner organisations’ operations. Reducing GHG emissions of organisations’ own operations is an important contribution to the race towards Net-Zero.</t>
+  </si>
+  <si>
+    <t>7F-07194.01</t>
+  </si>
+  <si>
+    <t>Maximum cooperation needed to manage glacier melt in Central Asia</t>
+  </si>
+  <si>
+    <t>How to meet the needs of Central Asias 68 million inhabitants for water while respecting the glaciers overlooking Kyrgyzstan, Tajikistan, Uzbekistan and Kazakhstan? The SDCs project is building on voluntary regional cooperation and rigorous scientific monitoring of the changes taking place in the glaciers.</t>
+  </si>
+  <si>
+    <t>7F-07324.06</t>
+  </si>
+  <si>
+    <t>Livelihoods and Food Security Fund - LIFT</t>
+  </si>
+  <si>
+    <t>The Livelihoods and Food Security Fund (LIFT) is a multi-donor fund, coordinating and contributing aid to rural development in Myanmar. Within its strategy period 2019-2023 LIFT will benefit 3.7 million additionl people with a strong focus on leaving no one behind, while working on more inclusive government policies and supporting the private sector. As chair for the LIFT Fund Board in the coming 12 months, Switzerland will ensure LIFTs conflict-sensitivity and benefit from additional access to key decision makers.</t>
+  </si>
+  <si>
+    <t>7F-07689.04.81</t>
+  </si>
+  <si>
+    <t>Water Security Middle East (Blue Peace)</t>
+  </si>
+  <si>
+    <t>In the Middle East, the dire situation of water resources demands stronger regional cooperation than ever before. The Blue Peace Middle East Initiative is the only regional platform engaging six countries around water issues. Together with its partners from academia, international organisations, civil society and the private sector, Switzerland is able to promote policy and concrete solutions for serving the most vulnerable populations leading to sustainable development and peace building. Stability in the region is in the interest of Switzerland.</t>
+  </si>
+  <si>
+    <t>7F-07801.03</t>
+  </si>
+  <si>
+    <t>Production des Connaissances et Appui Institutionnel pour une gestion intégrée des Ressources en Eau au Tchad - ResEau</t>
+  </si>
+  <si>
+    <t>Le Tchad subit fortement les effets du changement climatique avec des pluviométries aléatoires. Le sous-sol du Tchad dispose d’un important potentiel en eau. Faute de compétences nationales, ces ressources en eau restent très peu mobilisées. La DDC renforce, à travers ce projet, les compétences et les connaissances nationales pour favoriser une gestion durable de ces ressources et contribue ainsi à la résilience du Tchad face aux changements climatiques.</t>
+  </si>
+  <si>
+    <t>7F-07952.03</t>
+  </si>
+  <si>
+    <t>Swisscontact: Making Market Work for the Jamuna Padma and Teesta Chars M4C</t>
+  </si>
+  <si>
+    <t>Leveraging on Switzerlands longstanding engagement and experience in pro-poor agricultural market development, this project will benefit 75,000 poor and disadvantaged households living on riverine islands through profitable and environmentally sustainable livelihoods options. Thanks to improved access to agricultural inputs and services, access to output markets and financial services, they will generate an additional income of CHF 14.5 million to be invested into the diversification of their farm business and basic needs.</t>
+  </si>
+  <si>
+    <t>7F-08038.03</t>
+  </si>
+  <si>
+    <t>Gestion des Eaux de Ruissellement dans le Tchad Sahélien (GERTS)</t>
+  </si>
+  <si>
+    <t>Ce programme vise laménagement des vallées avec des seuils dépandage en vue de leur exploitation agro-pastorale au bénéfice direct de 350'000 personnes dans quatre régions au centre-est du Tchad. Cette approche est promue et mise à léchelle avec lappui dorganisations publiques et privées. Les femmes et les jeunes sont particulièrement encouragés à sinvestir en production maraîchère à but commercial et pour améliorer la nutrition. Le programme contribue aussi à la stabilité au centre-est du Tchad, et à la prévention de la migration et de lextrémisme violent.</t>
+  </si>
+  <si>
+    <t>7F-08245.03</t>
+  </si>
+  <si>
+    <t>PFNL - Programme d'appui à la valorisation des produits forestiers non ligneux au Burkina Faso</t>
+  </si>
+  <si>
+    <t>Au Burkina Faso, le fort potentiel en produits forestiers non ligneux peut être davantage exploité au profit des populations vulnérables en améliorant la sécurité alimentaire et la création de revenus. Pour une dernière phase, la Suisse, avec le cofinancement des Pays-Bas, consolide les acquis dune manière durable tout en soutenant lextension dans une nouvelle région pour prendre en compte, en particulier les personnes déplacées internes (PDI), les femmes et les jeunes affectés par la crise sécuritaire.</t>
+  </si>
+  <si>
+    <t>7F-08248.02.51</t>
+  </si>
+  <si>
+    <t>National Water Resources Management Project Ph 2</t>
+  </si>
+  <si>
+    <t>Water is not yet managed in a comprehensive manner in Kyrgyzstan and the national Water Code is not implemented. The project aims at supporting a structural reform and enhancing the capacities of water institutions to enable an effective implementation of the water code, which takes into account the various interests of all water users and the effects of climate change. Working on central governance issues, the results of this project will benefit to all other interventions related to water.</t>
+  </si>
+  <si>
+    <t>7F-08325.02.51</t>
+  </si>
+  <si>
+    <t>Municipal Environmental Governance (MEG)</t>
+  </si>
+  <si>
+    <t>Close to one quarter of the municipalities in the country will adopt a new performance management system, in line with the reforms of the public administration. Elected officials and municipal administrations will perform their duties and interact with citizens in a more responsive and transparent way. Citizens will benefit from better services, in particular in the water sector, in line with the European Union standards, and by developing synergies with the World Bank Water Supply and Sanitation Sector Modernization Programme. The regulatory framework at all levels will be improved to support these reforms.</t>
+  </si>
+  <si>
+    <t>7F-08361.02.51</t>
+  </si>
+  <si>
+    <t>Integrated Health and Habitat Improvement (IHHI) Rasht Valley</t>
+  </si>
+  <si>
+    <t>Through the project the population living in one of the poorest and fragile regions of Tajikistan (Rasht Valley) will gain access to basic social services (water and health). The interventions in the selected watersheds will empower the local communities enabling their active participation in decision-making and effective management of the resources. As a result, people in the project area will adopt healthier, more environmentally sustainable, and disaster-safer behaviours.</t>
+  </si>
+  <si>
+    <t>7F-08374.02.51</t>
+  </si>
+  <si>
+    <t>Potable Water Management Programme (PWMP) in Upper Egypt Phase 2</t>
+  </si>
+  <si>
+    <t>Egypt has critical needs in better managing water resources and reducing water losses as well as consumption, especially in Upper Egypt (climate change impact, lack of infrastructure, high poverty level). Switzerland provides innovative solutions for improved potable water management and service provision to the vulnerable population. The mixed approach based on strengthening capacities of the water company, improving the infrastructure for potable water provision and on engaging the communities will serve as model for nationwide replication.</t>
+  </si>
+  <si>
+    <t>7F-08496.02.54</t>
+  </si>
+  <si>
+    <t>Support for cooperative management in the agricultural sector in Cuba (APOCOOP)</t>
+  </si>
+  <si>
+    <t>APOCOOP contributes to food security in 17 municipalities by improving the management of agricultural cooperatives, strengthening tools and enhancing the capacities and conditions of cooperative members and other actors. It promotes models of inter-cooperation between agricultural cooperatives, with gender equity, resilience and economic, social and environmental sustainability, and to socialize results and methods in spaces of influence on land policies in Cuba.</t>
+  </si>
+  <si>
+    <t>7F-08580.02.51</t>
+  </si>
+  <si>
+    <t>Strengthening the Role of Local Communities in Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>The Project will enhance community governance in BiH by empowering local communities (MZs) as modern and effective structures for pro-active citizens participation. A new functional and organizational set up of MZs in BiH will be created and standardized countrywide. In turn, women and men will benefit from more people-centred local service delivery, better accountability and transparency of municipalities.</t>
+  </si>
+  <si>
+    <t>7F-08596.01.54</t>
+  </si>
+  <si>
+    <t>Bangladesh Agricultural and Disaster Insurance Programme (BADIP)</t>
+  </si>
+  <si>
+    <t>Smallholder farmers in Bangladesh face considerable risks. Droughts, floods, winds, temperature shocks, pests and diseases can destroy their livelihoods and leave them indebted for years. To cope with such shocks, they are often forced to sell productive assets and fall back in poverty. By developing the market for agricultural insurance and related extension services, BADIP will sustainably increase poor farmers resilience, giving them the confidence and security to step up their productive investments.</t>
+  </si>
+  <si>
+    <t>7F-08621.03.51</t>
+  </si>
+  <si>
+    <t>Modernization of Vocational Education and Training related to Agriculture in Georgia</t>
+  </si>
+  <si>
+    <t>Agricultural productivity and incomes are low in Georgia, which is largely due to obsolete knowledge and skills. The project contributes to introducing systemic changes in agriculture-related vocational education and extension services, increasing the role of private sector actors in planning and delivering vocational training. Rural youth, women and men, will thus be better trained and acquire more relevant skills; this will contribute to increasing their incomes and employment opportunities.</t>
+  </si>
+  <si>
+    <t>7F-08632.02</t>
+  </si>
+  <si>
+    <t>PIA-ACC - Applied Research Project for Climate Change Adaptation</t>
+  </si>
+  <si>
+    <t>Bolivia is highly vulnerable to the effects of Climate Change. Thus, scientific information needs to be generated and used to upscale the communities capacity for resilience. Universities are key players in the area of research and have the potential to support development. This project aims to strengthen the capacity and sustainability of the Bolivian university systems. Results shall be shared with public institutions to ensure greater adherence to and impact on public policy.</t>
+  </si>
+  <si>
+    <t>7F-08840.03.01</t>
+  </si>
+  <si>
+    <t>Programme de Valorisation du Potentiel Agro-Pastoral dans lEst du Burkina Faso (VALPAPE) Phase 3</t>
+  </si>
+  <si>
+    <t>La région de lEst du Burkina Faso est affectée par une grave crise sécuritaire et humanitaire qui risque dannihiler les bons résultats des dernières années sur le plan agropastoral. Aussi, la Suisse veut contribuer à la sauvegarde des acquis de développement tout en renforçant les moyens d'existence des personnes vulnérables touchées par des déplacements. En facilitant leur réinsertion socioéconomique, le programme participe à réduire leur vulnérabilité à lextrême pauvreté et à linsécurité alimentaire.</t>
+  </si>
+  <si>
+    <t>7F-08846.03</t>
+  </si>
+  <si>
+    <t>Lao Upland Rural Advisory Service (LURAS)</t>
+  </si>
+  <si>
+    <t>Laos is an agriculture-based country in transition. Farmers in the Northern region require additional knowledge, skills and access to resources to organize themselves within the ongoing agricultural socio-economic changes. Switzerlands expertise in inclusive economic development, climate change and environment will support rural advisory services during this final phase to sustainably stimulate climate resilient and lasting improvements in agricultural production and income generation for these farmers.</t>
+  </si>
+  <si>
+    <t>7F-08846.02.62</t>
+  </si>
+  <si>
+    <t>The rapid transformation of the rural economy brings smallholder farmers in contact with a wide range of new service providers (private agribusiness companies, farmer organisations, non-profit associations). The Ministry of Agriculture and Forestry (MAF) recognizes that greater pluralism in service provision is needed. LURAS supports a multi-stakeholder market-based approach to promote demand-driven service provision to farmers and strengthen the capacities of farmers’ organizations.</t>
+  </si>
+  <si>
+    <t>7F-08980.03</t>
+  </si>
+  <si>
+    <t>Strengthening Drought Resilience in the Somali National Regional State, Ethiopia (SDR-SNRS)</t>
+  </si>
+  <si>
+    <t>The livelihoods of pastoralists and agro-pastoralists in Somali National Regional State are increasingly threatened by environmental, socio-economic, and political upheavals. GIZ, in cooperation with Local Government partners, aims to build the resilience of vulnerable pastoralist communities through proven land rehabilitation measures, the promotion of livelihood activities, and capacity development of government and private sector institutions.</t>
+  </si>
+  <si>
+    <t>7F-09038.01</t>
+  </si>
+  <si>
+    <t>7F-09062.03.41</t>
+  </si>
+  <si>
+    <t>Contribution to Earth Security</t>
+  </si>
+  <si>
+    <t>This programme aims at catalysing new financial mechanisms and partnerships, including with the Swiss finance sector, which promote water-related ecosystem services of forests as a climate solution vital to the water cycle and to the benefit of society. While global in scope it will focus low and lower-middle income countries. It will leverage Swiss Know-How across the Federal Administration and contribute to the climate mainstreaming goal of the Dispatch 2021-24.</t>
+  </si>
+  <si>
+    <t>7F-09364.02</t>
+  </si>
+  <si>
+    <t>ENUFF - Enhancing Nutrition of Upland Farming Families</t>
+  </si>
+  <si>
+    <t>Despite a sustained economic growth of 7.7% over the last decade of Lao PDR, children under five, nationally, 21% are underweight, 33% are stunted and 9% wasted (2017). Based on initial achievements and lessons learned from phase one, Switzerland, with its leave no one behind value, will provide support for a second and final phase to the government­s multi-sectoral approach that integrates agriculture, nutrition, sanitation and hygiene. The geographical scope expands to 20 new remote villages and targets women, men and children.</t>
+  </si>
+  <si>
+    <t>7F-09393.02</t>
+  </si>
+  <si>
+    <t>Territorial water governance in the Gulf of Fonseca Region - phase II</t>
+  </si>
+  <si>
+    <t>The Program facilitates the empowerment of the Watershed Councils of the Nacaome, Choluteca and Sampile rivers in the Gulf of Fonseca Region in terms of their leadership and sustainable and participatory management of the water governance system. This contributes to collaborative processes and investments in the frame of the formulation and implementation of watershed plans, indirectly benefiting 500,000 inhabitants.</t>
+  </si>
+  <si>
+    <t>7F-09521.02</t>
+  </si>
+  <si>
+    <t>City Regions Food Systems (RUNRES)</t>
+  </si>
+  <si>
+    <t>Implemented by the Group of Sustainable Agroecosystems at ETHZ and local partners, RUNRES will improve the resilience of food systems in four different rural-urban regions across Africa. It will encourage organic and human waste recycling by implementing and scaling of viable innovations to transform waste into soil amendments or animal feed to serve as an input for agricultural production of smallholders, thereby contributing to food security, and human and environmental health in city region food systems.</t>
+  </si>
+  <si>
+    <t>7F-09609.02</t>
+  </si>
+  <si>
+    <t>REGLEAU - Renforcement de la gouvernance locale de leau et de lassainissement</t>
+  </si>
+  <si>
+    <t>Ce projet vise à renforcer les capacités de six communes dHaïti afin qu'elles puissent fournir des services d'eau potable et d'assainissement résilients aus risques et catastrophes à la population. En vue de la fin de la coopération bilatérale de la Suisse en Haïti, la phase II consolide et met à l'échelle les acquis de la première phase et intègre des approches du projet direct humanitaire « Réduction des Risques de Catastrophes Naturelles ».</t>
+  </si>
+  <si>
+    <t>7F-09710.01.51</t>
+  </si>
+  <si>
+    <t>ARCH Adaptive and Resilient Communities in their Habitat</t>
+  </si>
+  <si>
+    <t>The project aims at supporting the remote mountainous communities of Pamirs and authorities in developing resilient habitat and improving people's livelihoods in Tajikistan. This will be achieved through reducing vulnerabilities to natural hazards while strengthening participative disaster risk governance as well as joint definition and implementation of relevant risk reduction measures.</t>
+  </si>
+  <si>
+    <t>7F-09743.01</t>
+  </si>
+  <si>
+    <t>Diffusion des produits de la recherche agricole en Afrique de l’Ouest</t>
+  </si>
+  <si>
+    <t>Lutilisation des innovations et technologies sont indispensables pour accroitre la résilience et la productivité des systèmes alimentaires en Afrique de lOuest, en vue dy accroître leur adaptation aux changements climatiques et la sécurité alimentaire. La Suisse soutiendra le CORAF pour accroitre lutilisation par les producteurs, transformateurs et autres acteurs des chaines de valeurs agricoles des innovations produites par la recherche en soutenant leur diffusion et mutualisation.</t>
+  </si>
+  <si>
+    <t>7F-09748.01.51</t>
+  </si>
+  <si>
+    <t>IGGE : Inclusive Green Growth in Egypt</t>
+  </si>
+  <si>
+    <t>The main barriers to the competitiveness of the total 2.5 million micro-small-medium enterprises in Egypt are a lack of affordable funding and a mismatch between the needs of the market and the skills available. With its proven expertise in micro-small-medium enterprises Switzerland supports economic growth and more efficient use of resources in Upper Egypt through the model of green economy such as utilizing agricultural waste to create jobs and strengthen livelihoods of communities.</t>
+  </si>
+  <si>
+    <t>7F-09862.01</t>
+  </si>
+  <si>
+    <t>Inclusive Economic Development Program Territorial Region 13 Gulf of Fonseca</t>
+  </si>
+  <si>
+    <t>The program contributes to generate 5'000 new jobs and to increase the income of 10000 vulnerable families living in the watersheds of Choluteca, Goascorán and Nacaome by 10% annually. The program promotes public-private partnerships taking into account the challenges and potentials of smallholder families producing cashew, sustainable livestock and eco-tourism. It also facilitates territorial dialogue to establish rules that foster a business climate that combines financial benefits with social and environmental sustainability.</t>
+  </si>
+  <si>
+    <t>Strengthen local capacity</t>
+  </si>
+  <si>
+    <t>Research</t>
+  </si>
+  <si>
+    <t>Capacity building explicitally mentioned in description</t>
+  </si>
+  <si>
+    <t>No evident technology or research component</t>
+  </si>
+  <si>
+    <t>Not sure about capacity building</t>
+  </si>
+  <si>
+    <t>Clearly transfering technology in the building sector</t>
+  </si>
+  <si>
+    <t>Regional cooperation</t>
+  </si>
+  <si>
+    <t>Scientific monitoring</t>
+  </si>
+  <si>
+    <t>The project designs and promotes learning materials and supports national strategies. No specific technology is transferred</t>
+  </si>
+  <si>
+    <t>Strengthens human resources and skills (individual competencies and enabling environment). Clear capacity development.</t>
+  </si>
+  <si>
+    <t>Support to the African Forest Forum is knowledge and policy work reflected in NDCs. No technology is transferred, so TT is not marked.</t>
+  </si>
+  <si>
+    <t>Strengthens institutional and policy capacity (enabling environment).</t>
+  </si>
+  <si>
+    <t>Develops the market for agricultural insurance. No specific technology is transferred, so TT is not marked.</t>
+  </si>
+  <si>
+    <t>Market and financial-service development, not structured capacity development of institutions or individuals in the definitional sense.</t>
+  </si>
+  <si>
+    <t>Catalyses innovative financial mechanisms for ecosystem services. The TT finance clause applies only to finance at stages of the technology cycle; here finance supports ecosystem services, not a technology, so TT is not marked.</t>
+  </si>
+  <si>
+    <t>No structured capacity development is described.</t>
+  </si>
+  <si>
+    <t>introduces payments for ecosystem services, an innovative financing mechanism, but it finances a conservation outcome, not a technology cycle, so the TT finance clause does not apply. TT not marked.</t>
+  </si>
+  <si>
+    <t>Strengthens institutions and organisations for protected-area management (enabling environment).</t>
   </si>
 </sst>
 </file>
@@ -906,9 +1307,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1223,7 +1625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01F6AF3D-77FE-4DC4-9420-C8E1426AAA98}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
@@ -1246,10 +1648,10 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G1" t="s">
         <v>259</v>
-      </c>
-      <c r="G1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1260,7 +1662,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1269,10 +1671,10 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
+        <v>260</v>
+      </c>
+      <c r="G2" t="s">
         <v>261</v>
-      </c>
-      <c r="G2" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1292,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
+        <v>262</v>
+      </c>
+      <c r="G3" t="s">
         <v>263</v>
-      </c>
-      <c r="G3" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1315,10 +1717,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1329,7 +1731,7 @@
         <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1338,10 +1740,10 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1349,11 +1751,11 @@
         <v>82</v>
       </c>
       <c r="B6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C6" t="s">
         <v>231</v>
       </c>
-      <c r="C6" t="s">
-        <v>232</v>
-      </c>
       <c r="D6">
         <v>1</v>
       </c>
@@ -1361,22 +1763,22 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>266</v>
+      </c>
+      <c r="G6" t="s">
         <v>267</v>
-      </c>
-      <c r="G6" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" t="s">
         <v>176</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>177</v>
       </c>
-      <c r="C7" t="s">
-        <v>178</v>
-      </c>
       <c r="D7">
         <v>1</v>
       </c>
@@ -1384,10 +1786,10 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
+        <v>268</v>
+      </c>
+      <c r="G7" t="s">
         <v>269</v>
-      </c>
-      <c r="G7" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1398,7 +1800,7 @@
         <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1407,10 +1809,10 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
+        <v>270</v>
+      </c>
+      <c r="G8" t="s">
         <v>271</v>
-      </c>
-      <c r="G8" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1430,10 +1832,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
+        <v>272</v>
+      </c>
+      <c r="G9" t="s">
         <v>273</v>
-      </c>
-      <c r="G9" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1444,7 +1846,7 @@
         <v>74</v>
       </c>
       <c r="C10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1453,10 +1855,125 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
+        <v>274</v>
+      </c>
+      <c r="G10" t="s">
         <v>275</v>
       </c>
-      <c r="G10" t="s">
-        <v>276</v>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>399</v>
+      </c>
+      <c r="G11" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>401</v>
+      </c>
+      <c r="G12" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>403</v>
+      </c>
+      <c r="G13" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>405</v>
+      </c>
+      <c r="G14" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>407</v>
+      </c>
+      <c r="G15" t="s">
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -1465,8 +1982,662 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA84213E-690B-4121-99D4-362763A01E4D}">
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>394</v>
+      </c>
+      <c r="G2" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>295</v>
+      </c>
+      <c r="B6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C6" t="s">
+        <v>297</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C8" t="s">
+        <v>303</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>304</v>
+      </c>
+      <c r="B9" t="s">
+        <v>305</v>
+      </c>
+      <c r="C9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>398</v>
+      </c>
+      <c r="G9" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>307</v>
+      </c>
+      <c r="B10" t="s">
+        <v>308</v>
+      </c>
+      <c r="C10" t="s">
+        <v>309</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B11" t="s">
+        <v>311</v>
+      </c>
+      <c r="C11" t="s">
+        <v>312</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>313</v>
+      </c>
+      <c r="B12" t="s">
+        <v>314</v>
+      </c>
+      <c r="C12" t="s">
+        <v>315</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>316</v>
+      </c>
+      <c r="B13" t="s">
+        <v>317</v>
+      </c>
+      <c r="C13" t="s">
+        <v>318</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>319</v>
+      </c>
+      <c r="B14" t="s">
+        <v>320</v>
+      </c>
+      <c r="C14" t="s">
+        <v>321</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>322</v>
+      </c>
+      <c r="B15" t="s">
+        <v>323</v>
+      </c>
+      <c r="C15" t="s">
+        <v>324</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>325</v>
+      </c>
+      <c r="B16" t="s">
+        <v>326</v>
+      </c>
+      <c r="C16" t="s">
+        <v>327</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>328</v>
+      </c>
+      <c r="B17" t="s">
+        <v>329</v>
+      </c>
+      <c r="C17" t="s">
+        <v>330</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>331</v>
+      </c>
+      <c r="B18" t="s">
+        <v>332</v>
+      </c>
+      <c r="C18" t="s">
+        <v>333</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>334</v>
+      </c>
+      <c r="B19" t="s">
+        <v>335</v>
+      </c>
+      <c r="C19" t="s">
+        <v>336</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>337</v>
+      </c>
+      <c r="B20" t="s">
+        <v>338</v>
+      </c>
+      <c r="C20" t="s">
+        <v>339</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>340</v>
+      </c>
+      <c r="B21" t="s">
+        <v>341</v>
+      </c>
+      <c r="C21" t="s">
+        <v>342</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>346</v>
+      </c>
+      <c r="B22" t="s">
+        <v>347</v>
+      </c>
+      <c r="C22" t="s">
+        <v>348</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>349</v>
+      </c>
+      <c r="B23" t="s">
+        <v>350</v>
+      </c>
+      <c r="C23" t="s">
+        <v>351</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>392</v>
+      </c>
+      <c r="G23" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>352</v>
+      </c>
+      <c r="B24" t="s">
+        <v>353</v>
+      </c>
+      <c r="C24" t="s">
+        <v>354</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>355</v>
+      </c>
+      <c r="B25" t="s">
+        <v>356</v>
+      </c>
+      <c r="C25" t="s">
+        <v>357</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>358</v>
+      </c>
+      <c r="B26" t="s">
+        <v>356</v>
+      </c>
+      <c r="C26" t="s">
+        <v>359</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>360</v>
+      </c>
+      <c r="B27" t="s">
+        <v>361</v>
+      </c>
+      <c r="C27" t="s">
+        <v>362</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>363</v>
+      </c>
+      <c r="B28" t="s">
+        <v>217</v>
+      </c>
+      <c r="C28" t="s">
+        <v>218</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>367</v>
+      </c>
+      <c r="B29" t="s">
+        <v>368</v>
+      </c>
+      <c r="C29" t="s">
+        <v>369</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>370</v>
+      </c>
+      <c r="B30" t="s">
+        <v>371</v>
+      </c>
+      <c r="C30" t="s">
+        <v>372</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>373</v>
+      </c>
+      <c r="B31" t="s">
+        <v>374</v>
+      </c>
+      <c r="C31" t="s">
+        <v>375</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>376</v>
+      </c>
+      <c r="B32" t="s">
+        <v>377</v>
+      </c>
+      <c r="C32" t="s">
+        <v>378</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>379</v>
+      </c>
+      <c r="B33" t="s">
+        <v>380</v>
+      </c>
+      <c r="C33" t="s">
+        <v>381</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>382</v>
+      </c>
+      <c r="B34" t="s">
+        <v>383</v>
+      </c>
+      <c r="C34" t="s">
+        <v>384</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>385</v>
+      </c>
+      <c r="B35" t="s">
+        <v>386</v>
+      </c>
+      <c r="C35" t="s">
+        <v>387</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>388</v>
+      </c>
+      <c r="B36" t="s">
+        <v>389</v>
+      </c>
+      <c r="C36" t="s">
+        <v>390</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G36" xr:uid="{DA84213E-690B-4121-99D4-362763A01E4D}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4871F319-5628-401C-9985-1C2212EB50A9}">
-  <dimension ref="A1:E92"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.88671875" customWidth="1"/>
@@ -1490,7 +2661,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>55</v>
       </c>
@@ -1498,7 +2669,7 @@
         <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1507,7 +2678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>57</v>
       </c>
@@ -1515,7 +2686,7 @@
         <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1524,7 +2695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>58</v>
       </c>
@@ -1541,7 +2712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>61</v>
       </c>
@@ -1558,7 +2729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>63</v>
       </c>
@@ -1575,7 +2746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>68</v>
       </c>
@@ -1592,16 +2763,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" t="s">
         <v>236</v>
       </c>
-      <c r="C8" t="s">
-        <v>237</v>
-      </c>
       <c r="D8">
         <v>0</v>
       </c>
@@ -1609,7 +2780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>76</v>
       </c>
@@ -1617,7 +2788,7 @@
         <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1626,7 +2797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>78</v>
       </c>
@@ -1634,7 +2805,7 @@
         <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1643,7 +2814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>80</v>
       </c>
@@ -1660,15 +2831,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1677,7 +2848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>84</v>
       </c>
@@ -1694,7 +2865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>86</v>
       </c>
@@ -1702,7 +2873,7 @@
         <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1719,7 +2890,7 @@
         <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1728,7 +2899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>90</v>
       </c>
@@ -1745,7 +2916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>92</v>
       </c>
@@ -1753,7 +2924,7 @@
         <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -1762,7 +2933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
@@ -1770,7 +2941,7 @@
         <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1779,7 +2950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>96</v>
       </c>
@@ -1821,7 +2992,7 @@
         <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1830,7 +3001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>103</v>
       </c>
@@ -1847,7 +3018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>105</v>
       </c>
@@ -1881,7 +3052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>110</v>
       </c>
@@ -1898,7 +3069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>112</v>
       </c>
@@ -1915,15 +3086,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B27" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1932,7 +3103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>115</v>
       </c>
@@ -1966,7 +3137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>120</v>
       </c>
@@ -1983,7 +3154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>122</v>
       </c>
@@ -2000,7 +3171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>125</v>
       </c>
@@ -2008,7 +3179,7 @@
         <v>126</v>
       </c>
       <c r="C32" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2017,7 +3188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>127</v>
       </c>
@@ -2051,16 +3222,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B35" t="s">
+        <v>243</v>
+      </c>
+      <c r="C35" t="s">
         <v>244</v>
       </c>
-      <c r="C35" t="s">
-        <v>245</v>
-      </c>
       <c r="D35">
         <v>0</v>
       </c>
@@ -2068,7 +3239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
@@ -2076,7 +3247,7 @@
         <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -2085,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>135</v>
       </c>
@@ -2136,7 +3307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>143</v>
       </c>
@@ -2153,7 +3324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>146</v>
       </c>
@@ -2161,7 +3332,7 @@
         <v>147</v>
       </c>
       <c r="C41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -2170,7 +3341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>148</v>
       </c>
@@ -2178,7 +3349,7 @@
         <v>149</v>
       </c>
       <c r="C42" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -2187,7 +3358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>150</v>
       </c>
@@ -2212,7 +3383,7 @@
         <v>154</v>
       </c>
       <c r="C44" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -2229,7 +3400,7 @@
         <v>156</v>
       </c>
       <c r="C45" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -2238,15 +3409,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B46" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C46" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -2257,30 +3428,30 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B47" t="s">
         <v>159</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
+        <v>250</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C47" t="s">
-        <v>251</v>
-      </c>
-      <c r="D47">
-        <v>1</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+      <c r="B48" t="s">
         <v>161</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>162</v>
-      </c>
-      <c r="C48" t="s">
-        <v>163</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -2291,115 +3462,115 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B49" t="s">
         <v>164</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>165</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D49">
-        <v>1</v>
-      </c>
-      <c r="E49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+      <c r="B50" t="s">
         <v>167</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
+        <v>167</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C50" t="s">
-        <v>168</v>
-      </c>
-      <c r="D50">
-        <v>0</v>
-      </c>
-      <c r="E50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+      <c r="B51" t="s">
         <v>169</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
+        <v>169</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C51" t="s">
-        <v>170</v>
-      </c>
-      <c r="D51">
-        <v>0</v>
-      </c>
-      <c r="E51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+      <c r="B52" t="s">
         <v>171</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
+        <v>251</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C52" t="s">
+      <c r="B53" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" t="s">
+        <v>174</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C54" t="s">
+        <v>180</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B55" t="s">
         <v>252</v>
       </c>
-      <c r="D52">
-        <v>0</v>
-      </c>
-      <c r="E52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="B53" t="s">
-        <v>174</v>
-      </c>
-      <c r="C53" t="s">
-        <v>175</v>
-      </c>
-      <c r="D53">
-        <v>0</v>
-      </c>
-      <c r="E53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B54" t="s">
-        <v>180</v>
-      </c>
-      <c r="C54" t="s">
-        <v>181</v>
-      </c>
-      <c r="D54">
-        <v>0</v>
-      </c>
-      <c r="E54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>253</v>
-      </c>
-      <c r="C55" t="s">
-        <v>254</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -2410,47 +3581,47 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B56" t="s">
         <v>183</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
+        <v>254</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C56" t="s">
+      <c r="B57" t="s">
+        <v>185</v>
+      </c>
+      <c r="C57" t="s">
+        <v>185</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B58" t="s">
         <v>255</v>
       </c>
-      <c r="D56">
-        <v>1</v>
-      </c>
-      <c r="E56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B57" t="s">
-        <v>186</v>
-      </c>
-      <c r="C57" t="s">
-        <v>186</v>
-      </c>
-      <c r="D57">
-        <v>0</v>
-      </c>
-      <c r="E57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B58" t="s">
-        <v>256</v>
-      </c>
       <c r="C58" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -2461,149 +3632,149 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B59" t="s">
         <v>188</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>189</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-      <c r="E59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+      <c r="B60" t="s">
         <v>191</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
+        <v>223</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C60" t="s">
-        <v>224</v>
-      </c>
-      <c r="D60">
-        <v>0</v>
-      </c>
-      <c r="E60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
+      <c r="B61" t="s">
+        <v>256</v>
+      </c>
+      <c r="C61" t="s">
+        <v>223</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B62" t="s">
+        <v>194</v>
+      </c>
+      <c r="C62" t="s">
+        <v>195</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B63" t="s">
+        <v>197</v>
+      </c>
+      <c r="C63" t="s">
+        <v>198</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B64" t="s">
+        <v>200</v>
+      </c>
+      <c r="C64" t="s">
+        <v>223</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B65" t="s">
+        <v>202</v>
+      </c>
+      <c r="C65" t="s">
+        <v>203</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B66" t="s">
+        <v>205</v>
+      </c>
+      <c r="C66" t="s">
         <v>257</v>
       </c>
-      <c r="C61" t="s">
-        <v>224</v>
-      </c>
-      <c r="D61">
-        <v>0</v>
-      </c>
-      <c r="E61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B62" t="s">
-        <v>195</v>
-      </c>
-      <c r="C62" t="s">
-        <v>196</v>
-      </c>
-      <c r="D62">
-        <v>0</v>
-      </c>
-      <c r="E62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B63" t="s">
-        <v>198</v>
-      </c>
-      <c r="C63" t="s">
-        <v>199</v>
-      </c>
-      <c r="D63">
-        <v>0</v>
-      </c>
-      <c r="E63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B64" t="s">
-        <v>201</v>
-      </c>
-      <c r="C64" t="s">
-        <v>224</v>
-      </c>
-      <c r="D64">
-        <v>0</v>
-      </c>
-      <c r="E64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="B65" t="s">
-        <v>203</v>
-      </c>
-      <c r="C65" t="s">
-        <v>204</v>
-      </c>
-      <c r="D65">
-        <v>0</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B66" t="s">
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="C66" t="s">
-        <v>258</v>
-      </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-      <c r="E66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="B67" t="s">
         <v>6</v>
       </c>
       <c r="C67" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -2614,82 +3785,82 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B68" t="s">
         <v>209</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>210</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D68">
-        <v>1</v>
-      </c>
-      <c r="E68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
+      <c r="B69" t="s">
         <v>212</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>213</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D69">
-        <v>0</v>
-      </c>
-      <c r="E69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
+      <c r="B70" t="s">
         <v>215</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
+        <v>223</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="C70" t="s">
-        <v>224</v>
-      </c>
-      <c r="D70">
-        <v>0</v>
-      </c>
-      <c r="E70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
+      <c r="B71" t="s">
         <v>217</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>218</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D71">
-        <v>0</v>
-      </c>
-      <c r="E71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
+      <c r="B72" t="s">
         <v>220</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>221</v>
       </c>
-      <c r="C72" t="s">
-        <v>222</v>
-      </c>
       <c r="D72">
         <v>0</v>
       </c>
@@ -2697,7 +3868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>7</v>
       </c>
@@ -2714,7 +3885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>10</v>
       </c>
@@ -2731,7 +3902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>12</v>
       </c>
@@ -2748,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>14</v>
       </c>
@@ -2765,7 +3936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>16</v>
       </c>
@@ -2782,7 +3953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>18</v>
       </c>
@@ -2799,7 +3970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>20</v>
       </c>
@@ -2816,7 +3987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>25</v>
       </c>
@@ -2833,7 +4004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>28</v>
       </c>
@@ -2850,7 +4021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>30</v>
       </c>
@@ -2858,7 +4029,7 @@
         <v>31</v>
       </c>
       <c r="C82" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D82">
         <v>0</v>
@@ -2867,7 +4038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>32</v>
       </c>
@@ -2875,7 +4046,7 @@
         <v>33</v>
       </c>
       <c r="C83" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -2884,7 +4055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>34</v>
       </c>
@@ -2892,7 +4063,7 @@
         <v>35</v>
       </c>
       <c r="C84" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D84">
         <v>0</v>
@@ -2901,16 +4072,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B85" t="s">
+        <v>225</v>
+      </c>
+      <c r="C85" t="s">
         <v>226</v>
       </c>
-      <c r="C85" t="s">
-        <v>227</v>
-      </c>
       <c r="D85">
         <v>0</v>
       </c>
@@ -2918,7 +4089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>37</v>
       </c>
@@ -2935,7 +4106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>40</v>
       </c>
@@ -2952,7 +4123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>45</v>
       </c>
@@ -2960,7 +4131,7 @@
         <v>46</v>
       </c>
       <c r="C88" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D88">
         <v>0</v>
@@ -2969,7 +4140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>47</v>
       </c>
@@ -2977,7 +4148,7 @@
         <v>48</v>
       </c>
       <c r="C89" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D89">
         <v>0</v>
@@ -2986,7 +4157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>51</v>
       </c>
@@ -3003,7 +4174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>53</v>
       </c>
@@ -3011,7 +4182,7 @@
         <v>54</v>
       </c>
       <c r="C91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -3020,24 +4191,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B92" t="s">
-        <v>231</v>
-      </c>
-      <c r="C92" t="s">
-        <v>232</v>
-      </c>
-      <c r="D92">
-        <v>1</v>
-      </c>
-      <c r="E92">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:E91" xr:uid="{4871F319-5628-401C-9985-1C2212EB50A9}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>